<commit_message>
docs(readme): update Accounts.xlsx documentation with account type guidance
</commit_message>
<xml_diff>
--- a/Accounts.template.xlsx
+++ b/Accounts.template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="f:\Documents\Sync-Receipts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D39D6845-E2D3-4931-A30A-D23E9891E9E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF23BA24-4DC4-4A5D-8DFF-B123AB83CA7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C2EC8488-05C0-43B5-B75B-E4C4A895CE3B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="16">
   <si>
     <t>Last 4</t>
   </si>
@@ -53,9 +53,6 @@
     <t>Type</t>
   </si>
   <si>
-    <t>1234</t>
-  </si>
-  <si>
     <t>John Doe</t>
   </si>
   <si>
@@ -68,22 +65,25 @@
     <t>Credit</t>
   </si>
   <si>
-    <t>4455</t>
-  </si>
-  <si>
     <t>Jane Doe</t>
   </si>
   <si>
-    <t>My Credit Union</t>
-  </si>
-  <si>
     <t>Checking</t>
   </si>
   <si>
-    <t>0000</t>
-  </si>
-  <si>
     <t>Cash</t>
+  </si>
+  <si>
+    <t>Mastercard</t>
+  </si>
+  <si>
+    <t>Debit</t>
+  </si>
+  <si>
+    <t>Savings</t>
+  </si>
+  <si>
+    <t>EBT</t>
   </si>
 </sst>
 </file>
@@ -466,13 +466,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03E5C2F5-63F0-42D4-9A84-DF7543A3E423}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -494,30 +494,33 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2">
+        <v>1234</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>10</v>
+      <c r="A3">
+        <v>5678</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
         <v>12</v>
       </c>
       <c r="E3" t="s">
@@ -525,15 +528,66 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4">
+        <v>6310</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>6310</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s">
         <v>14</v>
       </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" t="s">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>943</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
         <v>15</v>
       </c>
+      <c r="E6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>0</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
chore(accounts): format Accounts.template.xlsx as Excel table (TableStyleMedium2)
</commit_message>
<xml_diff>
--- a/Accounts.template.xlsx
+++ b/Accounts.template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="f:\Documents\Sync-Receipts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF23BA24-4DC4-4A5D-8DFF-B123AB83CA7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{23AED375-DA43-4F13-A5CD-AB99667C0C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C2EC8488-05C0-43B5-B75B-E4C4A895CE3B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CBA46100-9164-42DE-B79D-BCBCEC8B08F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Accounts" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
   <si>
     <t>Last 4</t>
   </si>
@@ -53,6 +53,9 @@
     <t>Type</t>
   </si>
   <si>
+    <t>1234</t>
+  </si>
+  <si>
     <t>John Doe</t>
   </si>
   <si>
@@ -65,41 +68,45 @@
     <t>Credit</t>
   </si>
   <si>
+    <t>5678</t>
+  </si>
+  <si>
+    <t>Mastercard</t>
+  </si>
+  <si>
+    <t>Debit</t>
+  </si>
+  <si>
+    <t>6310</t>
+  </si>
+  <si>
+    <t>Checking</t>
+  </si>
+  <si>
+    <t>Savings</t>
+  </si>
+  <si>
+    <t>0943</t>
+  </si>
+  <si>
     <t>Jane Doe</t>
   </si>
   <si>
-    <t>Checking</t>
+    <t>EBT</t>
+  </si>
+  <si>
+    <t>0000</t>
   </si>
   <si>
     <t>Cash</t>
-  </si>
-  <si>
-    <t>Mastercard</t>
-  </si>
-  <si>
-    <t>Debit</t>
-  </si>
-  <si>
-    <t>Savings</t>
-  </si>
-  <si>
-    <t>EBT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -127,16 +134,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -147,6 +156,20 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{50309A1C-B440-4A59-8CE6-73E87C578C87}" name="Accounts" displayName="Accounts" ref="A1:E7" totalsRowShown="0">
+  <autoFilter ref="A1:E7" xr:uid="{50309A1C-B440-4A59-8CE6-73E87C578C87}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{1EB8C79E-FC90-465D-8868-1F043F162229}" name="Last 4" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{96F63431-C3B1-47B4-9374-945E3C9B425A}" name="Holder"/>
+    <tableColumn id="3" xr3:uid="{3F67CA97-4731-479F-8F5B-1D974FC709D1}" name="Institution"/>
+    <tableColumn id="4" xr3:uid="{09C18D87-349A-4EDD-90CE-A7C5A4B115A0}" name="Network"/>
+    <tableColumn id="5" xr3:uid="{844ADA0F-183E-4348-87B7-4052A77188E2}" name="Type"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -465,131 +488,125 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03E5C2F5-63F0-42D4-9A84-DF7543A3E423}">
-  <dimension ref="A1:E10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CCB5D12-F6A7-47F5-92E8-B7EC76E1230A}">
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1234</v>
+      <c r="A2" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>5678</v>
+      <c r="A3" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
         <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>6310</v>
+      <c r="A4" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>6310</v>
+      <c r="A5" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>943</v>
+      <c r="A6" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>0</v>
+      <c r="A7" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10"/>
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>